<commit_message>
verify sheet export import column names updated
</commit_message>
<xml_diff>
--- a/AdvanceCRM/AdvanceCRM.Web/Templates/MasterSupression_Template.xlsx
+++ b/AdvanceCRM/AdvanceCRM.Web/Templates/MasterSupression_Template.xlsx
@@ -17,10 +17,10 @@
     <t>Sr No</t>
   </si>
   <si>
-    <t>Account Number</t>
+    <t>Master Account ID</t>
   </si>
   <si>
-    <t>Campaign Id</t>
+    <t>Campaign ID</t>
   </si>
   <si>
     <t>Company Name</t>

</xml_diff>